<commit_message>
dados: estado e planilhas do reprocessamento, auditoria, consolidado e insumos locais
</commit_message>
<xml_diff>
--- a/saida/produtos_enriquecidos_parte_1.xlsx
+++ b/saida/produtos_enriquecidos_parte_1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45634,12 +45634,12 @@
       </c>
       <c r="G870" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Largura da lâmina: 2,5 cm; Comprimento: 254 mm; Material: Aço especial forjado e termicamente tratado; Peso: 0,536 Kg/Un.</t>
         </is>
       </c>
       <c r="H870" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.mercadolivre.com.br/talhadeira-sao-romao-chata-10/up/MLBU3137308650</t>
         </is>
       </c>
       <c r="I870" t="inlineStr">
@@ -45647,7 +45647,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J870" t="inlineStr"/>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>https://www.saoromao.com.br/wp-content/uploads/2015/04/TALHADEIRA-A%C3%87O-LISO-S%C3%83O-ROM%C3%83O.png</t>
+        </is>
+      </c>
     </row>
     <row r="871">
       <c r="A871" t="inlineStr">
@@ -45826,12 +45830,12 @@
       </c>
       <c r="G874" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Material: Aço de pó metalúrgico; Diâmetro externo: 50 mm, para tubo PVC 32 mm 1/2.</t>
         </is>
       </c>
       <c r="H874" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.ranova.com.br/ferramentas/ferramentas-diversas/tarraxa-rapida-ppvc-meikon</t>
         </is>
       </c>
       <c r="I874" t="inlineStr">
@@ -45839,7 +45843,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J874" t="inlineStr"/>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>https://images.tcdn.com.br/img/img_prod/1239768/tarraxa_rapida_1_2_meikon_9047_1_016825bfa152611c809eeb1fcdfbbc6f.jpeg | https://http2.mlstatic.com/D_NQ_NP_727268-MLU76746168357_052024-O.webp | https://cdn.awsli.com.br/600x1000/2506/2506129/produto/1792743054ca6e6382b.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="875">
       <c r="A875" t="inlineStr">
@@ -45872,14 +45880,10 @@
           <t>Tarracha rápida da marca Meikon, modelo 3/4.</t>
         </is>
       </c>
-      <c r="G875" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G875" t="inlineStr"/>
       <c r="H875" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.compensamais.com.br/produto/tarraxa-luva-rapida-para-tubos-3-4-meikon-72258</t>
         </is>
       </c>
       <c r="I875" t="inlineStr">
@@ -45887,7 +45891,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J875" t="inlineStr"/>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>https://compensamateriais.fbitsstatic.net/img/p/tarraxa-luva-rapida-para-tubos-3-4-meikon-72258/258777.jpg?w=640&amp;h=640&amp;v=no-change&amp;qs=ignore | https://compensamateriais.fbitsstatic.net/img/p/tarraxa-luva-rapida-para-tubos-3-4-meikon-72258/258777-1.jpg?w=640&amp;h=640&amp;v=no-change&amp;qs=ignore | https://compensamateriais.fbitsstatic.net/img/p/tarraxa-luva-rapida-para-tubos-3-4-meikon-72258/258777-2.jpg?w=640&amp;h=640&amp;v=no-change&amp;qs=ignore</t>
+        </is>
+      </c>
     </row>
     <row r="876">
       <c r="A876" t="inlineStr">
@@ -45922,12 +45930,12 @@
       </c>
       <c r="G876" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Dimensões (C x L x A): 63 x 16 x 3 centímetros, Peso: 2.50 Kg, Material: Aço carbono, Capacidade: Corta vergalhão de 10mm e 8mm</t>
         </is>
       </c>
       <c r="H876" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.mercadolivre.com.br/tesoura-manual-corta-vergalhao-24---mtx/up/MLBU1594168503</t>
         </is>
       </c>
       <c r="I876" t="inlineStr">
@@ -45935,7 +45943,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J876" t="inlineStr"/>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>https://a-static.mlcdn.com.br/90x90/tesoura-manual-para-cortar-vergalhao-24-pol-vonder/siriusweb/887/51d8d9e500ef7a6ce4a211058a098cbb.jpeg | https://a-static.mlcdn.com.br/90x90/tesoura-manual-para-cortar-vergalhao-24-pol-vonder/siriusweb/887/1a2f6968e9a229f23f8827640f0fbbee.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="877">
       <c r="A877" t="inlineStr">
@@ -46018,12 +46030,12 @@
       </c>
       <c r="G878" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Dimensões (C x L x A): 92 x 19 x 4 cm, Peso: 5.78 kg, Diâmetro da barra (aço macio): 16mm, Diâmetro da barra (aço maciço): 11mm</t>
         </is>
       </c>
       <c r="H878" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.magaluempresas.com.br/tesoura-manual-para-cortar-vergalhao-36-pol-785559-mtx-000770/p/je4j69ga8e/fs/tcvo?recommendation_id=7&amp;ads_metadata=</t>
         </is>
       </c>
       <c r="I878" t="inlineStr">
@@ -46031,7 +46043,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J878" t="inlineStr"/>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>https://a-static.mlcdn.com.br/400x600/tesoura-manual-para-cortar-vergalhao-36-pol-785559-mtx-000770/palaciodas-ferramentas/55186/0bf4b88496934f97fd21712ec7aea936.jpeg | https://luitex.vtexassets.com/arquivos/ids/167166-800-auto?v=637879533537600000&amp;width=800&amp;height=auto&amp;aspect=true</t>
+        </is>
+      </c>
     </row>
     <row r="879">
       <c r="A879" t="inlineStr">
@@ -46066,12 +46082,12 @@
       </c>
       <c r="G879" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Comprimento: 42 polegadas. Material das Lâminas: Aço Cromo Vanádio (CR V), proporcionando alta resistência e durabilidade. Aplicação: Indicada para cortes de vergalhões, parafusos, pinos e outros materiais similares.</t>
         </is>
       </c>
       <c r="H879" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.casadasoldablu.com.br/product-page/tesoura-corta-vergalh%C3%A3o-42-polegadas-worker</t>
         </is>
       </c>
       <c r="I879" t="inlineStr">
@@ -46079,7 +46095,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J879" t="inlineStr"/>
+      <c r="J879" t="inlineStr">
+        <is>
+          <t>https://images.tcdn.com.br/img/img_prod/794025/tesoura_corta_vergalhao_42_104_0005_1017789_1_9fe85f7a0a0215be3060a0b16df5ca87.jpg | https://images.tcdn.com.br/img/img_prod/794025/tesoura_corta_vergalhao_42_104_0005_1017789_2_7322ba9eefc78066dc48e193f98c8d74.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="880">
       <c r="A880" t="inlineStr">
@@ -46256,11 +46276,7 @@
           <t>Tesoura para cortar chapa de aviação.</t>
         </is>
       </c>
-      <c r="G883" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G883" t="inlineStr"/>
       <c r="H883" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -46352,11 +46368,7 @@
           <t>Tesoura para cortar grama, ideal para jardins e áreas verdes.</t>
         </is>
       </c>
-      <c r="G885" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G885" t="inlineStr"/>
       <c r="H885" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -46640,11 +46652,7 @@
           <t>Torno de bancada fixo, modelo 5, utilizado para trabalhos de precisão em oficinas e indústrias.</t>
         </is>
       </c>
-      <c r="G891" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G891" t="inlineStr"/>
       <c r="H891" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -46652,10 +46660,14 @@
       </c>
       <c r="I891" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
-      <c r="J891" t="inlineStr"/>
+          <t>https://pt.scribd.com/document/899067426/MR-325-1100W-MOTOR-BRUSHLESS-11-2023</t>
+        </is>
+      </c>
+      <c r="J891" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_NQ_NP_896161-MLA99602233012_122025-O.webp | https://www.dutramaquinas.com.br/shared/img/produto/alta/551445_torno_de_bancada_fixo_n_5_lider.jpg | https://ferramentasgerais.vteximg.com.br/arquivos/ids/1017689-292-292/Torno-de-bancada-n%C2%BA-5-mordentes-fixos-em-ferro-nodular-MR-5-MARCON---MR-5---MARCON.jpg?v=638929456906000000</t>
+        </is>
+      </c>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
@@ -46690,7 +46702,7 @@
       </c>
       <c r="G892" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Capacidade: 6 polegadas, Mordente fixo, Material: Aço</t>
         </is>
       </c>
       <c r="H892" t="inlineStr">
@@ -46703,7 +46715,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J892" t="inlineStr"/>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>https://anhangueraferramentas.fbitsstatic.net/img/p/torno-de-bancada-fixo-6-mr-6-92812/281239-2.jpg?w=460&amp;h=460&amp;v=no-value | https://anhangueraferramentas.fbitsstatic.net/img/p/torno-morsa-de-bancada-2-mordente-fixo-e-ferro-nodular-pratiko-schulz-120647/309897.jpg?w=460&amp;h=460&amp;v=no-value | https://anhangueraferramentas.fbitsstatic.net/img/p/torno-de-bancada-fixo-6-com-mordente-fixo-33890006-forjasul-133560/323257-3.jpg?w=650&amp;h=650&amp;v=no-value</t>
+        </is>
+      </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
@@ -46880,11 +46896,7 @@
           <t>TORQUES 8" - ferramenta de trabalho manual, provavelmente utilizada para apertar ou soltar parafusos e porcas.</t>
         </is>
       </c>
-      <c r="G896" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G896" t="inlineStr"/>
       <c r="H896" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -46895,7 +46907,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J896" t="inlineStr"/>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>https://ferramentasgerais.vteximg.com.br/arquivos/ids/995036-292-292/Torques-para-Carpinteiro-8---VONDER---3633008000---VONDER.jpg?v=638929289348230000 | https://static.lojabrafer.com.br/public/brafer/imagens/produtos/torques-carpinteiro-8-pol-cabo-emborrachado-mister-42031.jpg | https://ferramentasgerais.vteximg.com.br/arquivos/ids/1009214-292-292/Torques-Carpinteiro-8---41050-108---TRAMONTINA-MASTER.jpg?v=638929394363170000</t>
+        </is>
+      </c>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
@@ -46928,11 +46944,7 @@
           <t>O TORQUES 10'' é um produto cujas informações não puderam ser obtidas devido a um erro na busca na web.</t>
         </is>
       </c>
-      <c r="G897" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G897" t="inlineStr"/>
       <c r="H897" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -46943,7 +46955,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J897" t="inlineStr"/>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>https://ferramentasgerais.vteximg.com.br/arquivos/ids/963768-292-292/Torques-Armador-10---Gedore---8380-250---GEDORE.jpg?v=638918516854500000 | https://http2.mlstatic.com/D_NQ_NP_687928-MLA99622233460_122025-O.webp | https://http2.mlstatic.com/D_NQ_NP_732323-MLU73288325364_122023-O.webp</t>
+        </is>
+      </c>
     </row>
     <row r="898">
       <c r="A898" t="inlineStr">
@@ -46978,12 +46994,12 @@
       </c>
       <c r="G898" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Medida: 12 polegadas, Código: 000757</t>
         </is>
       </c>
       <c r="H898" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://hfferramentas.com/loja/torques-armador-000757-12/</t>
         </is>
       </c>
       <c r="I898" t="inlineStr">
@@ -46991,7 +47007,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J898" t="inlineStr"/>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>https://hfferramentas.com/wp-content/uploads/2023/11/Torque-armador.jpg | https://hfferramentas.com/wp-content/uploads/2023/11/Torque-armador-embalagem.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="899">
       <c r="A899" t="inlineStr">
@@ -47024,11 +47044,7 @@
           <t>TORQUES 5'', um produto cujas informações específicas não foram encontradas.</t>
         </is>
       </c>
-      <c r="G899" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G899" t="inlineStr"/>
       <c r="H899" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -47036,7 +47052,7 @@
       </c>
       <c r="I899" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://s3.us-east-1.amazonaws.com/hytorc-prod-libraryhytorc-webassets/8204/HYTORC-LST-Basic_Operations_Manual-PT-EMAIL.pdf</t>
         </is>
       </c>
       <c r="J899" t="inlineStr"/>
@@ -47069,22 +47085,22 @@
       </c>
       <c r="F900" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>O TORQUES 6'' é uma ferramenta elétrica de torque da família Lithium Series da HYTORC, projetada para aplicações industriais de alta precisão e confiabilidade.</t>
         </is>
       </c>
       <c r="G900" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Voltagem: 36V, Certificações: EN ISO 12100-1:2011, EN ISO 12100-2:2011, EN ISO 14121-1:2007, EN ISO 11148-6:2012, UL STDS 60745-1 &amp; 60745-2-2, CSA STD C22.2 Nos. 60745-1 &amp; 60745-2-2</t>
         </is>
       </c>
       <c r="H900" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.torquegun.com</t>
         </is>
       </c>
       <c r="I900" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://s3.us-east-1.amazonaws.com/hytorc-prod-libraryhytorc-webassets/7867/HYTORC-LITHIUM_SERIES-Operations_Manual-071420-PT.pdf</t>
         </is>
       </c>
       <c r="J900" t="inlineStr"/>
@@ -47405,17 +47421,17 @@
       </c>
       <c r="F907" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Jogo de macho manual de 1/2 polegada, composto por 3 peças, fabricado em aço liga, ideal para criar roscas internas em metais e ligas industriais.</t>
         </is>
       </c>
       <c r="G907" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Bitola: 1/2'', FPP: 13, Comprimento Total: 80mm, Comprimento Rosca: 29mm, Diâmetro Haste: 9mm, Diâmetro Broca: 10,7mm</t>
         </is>
       </c>
       <c r="H907" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.superproatacado.com.br/jogo-de-macho-manual-din351-unc-1-2-x13-3-pecas-worker-991830/p</t>
         </is>
       </c>
       <c r="I907" t="inlineStr">
@@ -47423,7 +47439,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J907" t="inlineStr"/>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>https://cdn.superproatacado.com.br/storage/superproatacado/1000/jogo-de-macho-manual-din351-unc-12x13-3-pecas-worker17696853091206271.jpeg | https://cdn.superproatacado.com.br/storage/superproatacado/1000/jogo-de-macho-manual-din351-unc-12x13-3-pecas-worker17696853098825782.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="908">
       <c r="A908" t="inlineStr">
@@ -47451,16 +47471,8 @@
           <t>MACHO</t>
         </is>
       </c>
-      <c r="F908" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
-      <c r="G908" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="F908" t="inlineStr"/>
+      <c r="G908" t="inlineStr"/>
       <c r="H908" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -47504,11 +47516,7 @@
           <t>MACHO WW AC 5/16 * é um componente de conexão, provavelmente usado em aplicações de engenharia ou construção.</t>
         </is>
       </c>
-      <c r="G909" t="inlineStr">
-        <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
+      <c r="G909" t="inlineStr"/>
       <c r="H909" t="inlineStr">
         <is>
           <t>Não encontrado</t>
@@ -48082,12 +48090,12 @@
       </c>
       <c r="G921" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Material do Carretel: Plástico com revestimento de borracha, Comprimento da Linha: 30 metros, Quantidade de Giz: 115g na cor azul</t>
         </is>
       </c>
       <c r="H921" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.mercadolivre.com.br/kit-linha-de-marcacao-30m--giz-em-po-azul-110g-bestfer/up/MLBU2344522248</t>
         </is>
       </c>
       <c r="I921" t="inlineStr">
@@ -48095,7 +48103,11 @@
           <t>Não encontrado</t>
         </is>
       </c>
-      <c r="J921" t="inlineStr"/>
+      <c r="J921" t="inlineStr">
+        <is>
+          <t>https://http2.mlstatic.com/D_Q_NP_2X_952910-MLB93639298108_102025-P.webp | https://http2.mlstatic.com/D_NQ_NP_646050-MLB106318433849_012026-O-giz-linha-marcacao-azul-30m-kit-irwin-gesso-drywall-obra.webp | https://http2.mlstatic.com/D_NQ_NP_949991-MLB84803518689_052025-O-kit-linha-de-marcacao-30m-giz-azul-bfh2912-bestfer.webp</t>
+        </is>
+      </c>
     </row>
     <row r="922">
       <c r="A922" t="inlineStr">
@@ -48322,20 +48334,24 @@
       </c>
       <c r="G926" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>Auto nivelamento em até 4 graus, alcance de trabalho interior de 30 m, emite 1 viga verde horizontal 360° e 2 vigas verdes verticais 360°, bateria recarregável, inclui baterias de lítio, carregador de baterias, micro USB, tripé e estojo de armazenamento.</t>
         </is>
       </c>
       <c r="H926" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>https://www.magazineluiza.com.br/nivel-a-laser-com-prumo-e-marker-10m-mtx-350069/p/ak7gc1ea80/fs/nala/</t>
         </is>
       </c>
       <c r="I926" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
-        </is>
-      </c>
-      <c r="J926" t="inlineStr"/>
+          <t>https://d7rh5s3nxmpy4.cloudfront.net/CMP5386/files/TLL255245_PT.pdf</t>
+        </is>
+      </c>
+      <c r="J926" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/61G3KQ49LTL.jpg | https://a-static.mlcdn.com.br/420x420/nivel-a-laser-com-prumo-marker-e-esquadro-mtx/ferramentacerta/628255584/2cdf6ad3b3e248a7e47903e4e2dfac8a.jpg | https://m.media-amazon.com/images/I/61-ap4Gg2nL.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="927">
       <c r="A927" t="inlineStr">

</xml_diff>